<commit_message>
Ingest SpaceX conference monetization guidance with scope safeguards
</commit_message>
<xml_diff>
--- a/data/ai-compute-economics.xlsx
+++ b/data/ai-compute-economics.xlsx
@@ -2,13 +2,13 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R2bb738fd055e4ec1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Company Models" sheetId="2" r:id="R91662472ea794b65"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Methods" sheetId="3" r:id="R7e0ae63a5d3e43cd"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Token Economics" sheetId="4" r:id="R547c56ca4fe148da"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Benchmarks" sheetId="5" r:id="Raccee738f57f45e4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="6" r:id="R1329e384db754b40"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Read Me" sheetId="7" r:id="Rc845151a41b24813"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R1e62ba5d08a44ce7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Company Models" sheetId="2" r:id="R8b00635d9fc44b9c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Methods" sheetId="3" r:id="Re6620be9f68447b6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Token Economics" sheetId="4" r:id="R7267c0535ffb48d9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Benchmarks" sheetId="5" r:id="Rd0b70d9d56e7403c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="6" r:id="Rdf125edc0fcd412a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Read Me" sheetId="7" r:id="R1b81a77c6f0c4873"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -362,7 +362,7 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="SourceRegisterTable" displayName="SourceRegisterTable" ref="A4:I13" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="SourceRegisterTable" displayName="SourceRegisterTable" ref="A4:I16" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="9">
     <x:tableColumn id="1" name="Source ID"/>
     <x:tableColumn id="2" name="Date"/>
@@ -989,14 +989,14 @@
       </x:c>
       <x:c r="D22" s="19" t="str">
         <x:f>'Company Models'!N14</x:f>
-        <x:v>CAPEX ONLY</x:v>
+        <x:v>GUIDANCE ONLY</x:v>
       </x:c>
       <x:c r="E22" s="58" t="str">
         <x:f>IF('Company Models'!S14="","",'Company Models'!S14)</x:f>
       </x:c>
       <x:c r="F22" s="19" t="str">
         <x:f>'Company Models'!T14</x:f>
-        <x:v>Not an operator output</x:v>
+        <x:v>Missing numerator or denominator</x:v>
       </x:c>
     </x:row>
     <x:row r="23">
@@ -1702,10 +1702,10 @@
         <x:v>SRC-WB-P2S-001</x:v>
       </x:c>
       <x:c r="N14" s="19" t="str">
-        <x:v>CAPEX ONLY</x:v>
+        <x:v>GUIDANCE ONLY</x:v>
       </x:c>
       <x:c r="O14" s="43" t="str">
-        <x:v>Revenue numerator not disclosed; power used for capex benchmark only</x:v>
+        <x:v>Capex power anchor only; Sep 10 guidance is $30-50B per stated GW-year; effective denominator unresolved</x:v>
       </x:c>
       <x:c r="P14" s="37" t="str">
         <x:f>IF(OR(D14="",E14="",F14=""),"",D14*E14*F14)</x:f>
@@ -1722,7 +1722,7 @@
       </x:c>
       <x:c r="T14" s="25" t="str">
         <x:f>IF(S14&lt;&gt;"","Calculated",IF(OR(N14="VENDOR ONLY",N14="CAPEX ONLY"),"Not an operator output","Missing numerator or denominator"))</x:f>
-        <x:v>Not an operator output</x:v>
+        <x:v>Missing numerator or denominator</x:v>
       </x:c>
     </x:row>
     <x:row r="15">
@@ -2181,16 +2181,16 @@
         <x:v>Reference operator</x:v>
       </x:c>
       <x:c r="D14" s="43" t="str">
-        <x:v>External compute revenue when disclosed</x:v>
+        <x:v>Recognized external compute revenue when reconciled</x:v>
       </x:c>
       <x:c r="E14" s="43" t="str">
         <x:v>Average effective Colossus IT MW</x:v>
       </x:c>
       <x:c r="F14" s="43" t="str">
-        <x:v>Reconcile capex PP&amp;E and CIP overlap; brownfield</x:v>
+        <x:v>Retain capex benchmark; separate Sep 10 monetization guidance until power scope reconciled</x:v>
       </x:c>
       <x:c r="G14" s="43" t="str">
-        <x:v>Capex anchor only</x:v>
+        <x:v>Capex anchor plus management guidance</x:v>
       </x:c>
     </x:row>
     <x:row r="15">
@@ -2265,7 +2265,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9ba8100367fc4aed"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc16d947a88b04b35"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2889,7 +2889,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf8afe7c2c5504bb2"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rcd47c55e6d8340dd"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3590,38 +3590,123 @@
       </x:c>
     </x:row>
     <x:row r="13">
-      <x:c r="A13" s="20" t="str">
+      <x:c r="A13" s="19" t="str">
         <x:v>SRC-NVDA-Q2FY27-001</x:v>
       </x:c>
-      <x:c r="B13" s="46" t="n">
+      <x:c r="B13" s="45" t="n">
         <x:v>46260</x:v>
       </x:c>
-      <x:c r="C13" s="20" t="str">
+      <x:c r="C13" s="19" t="str">
         <x:v>NVIDIA</x:v>
       </x:c>
-      <x:c r="D13" s="44" t="str">
+      <x:c r="D13" s="43" t="str">
         <x:v>Q2 FY2027 earnings call</x:v>
       </x:c>
-      <x:c r="E13" s="44" t="str">
+      <x:c r="E13" s="43" t="str">
         <x:v>Transcript</x:v>
       </x:c>
-      <x:c r="F13" s="44" t="str">
+      <x:c r="F13" s="43" t="str">
         <x:v>https://investor.nvidia.com/</x:v>
       </x:c>
-      <x:c r="G13" s="44" t="str">
+      <x:c r="G13" s="43" t="str">
         <x:v>Hopper Blackwell and Rubin content per GW</x:v>
       </x:c>
-      <x:c r="H13" s="44" t="str">
+      <x:c r="H13" s="43" t="str">
         <x:v>Primary</x:v>
       </x:c>
-      <x:c r="I13" s="44" t="str">
+      <x:c r="I13" s="43" t="str">
         <x:v>Exact transcript URL to pin on refresh</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="14">
+      <x:c r="A14" s="19" t="str">
+        <x:v>SRC-XAI-GS-RECAP-20260910</x:v>
+      </x:c>
+      <x:c r="B14" s="45" t="n">
+        <x:v>46275</x:v>
+      </x:c>
+      <x:c r="C14" s="19" t="str">
+        <x:v>User-supplied Goldman recap</x:v>
+      </x:c>
+      <x:c r="D14" s="43" t="str">
+        <x:v>SpaceX CFO Communacopia recap</x:v>
+      </x:c>
+      <x:c r="E14" s="43" t="str">
+        <x:v>Project message</x:v>
+      </x:c>
+      <x:c r="F14" s="43"/>
+      <x:c r="G14" s="43" t="str">
+        <x:v>Monetization guidance and capacity targets</x:v>
+      </x:c>
+      <x:c r="H14" s="43" t="str">
+        <x:v>Attributed recap</x:v>
+      </x:c>
+      <x:c r="I14" s="43" t="str">
+        <x:v>Raw recap in raw/2026-09-10-spacex-goldman-recap.md</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="15">
+      <x:c r="A15" s="19" t="str">
+        <x:v>SRC-XAI-GS-QA-20260910</x:v>
+      </x:c>
+      <x:c r="B15" s="45" t="n">
+        <x:v>46275</x:v>
+      </x:c>
+      <x:c r="C15" s="19" t="str">
+        <x:v>Bret Johnsen via Investing.com</x:v>
+      </x:c>
+      <x:c r="D15" s="43" t="str">
+        <x:v>SpaceX Communacopia full Q&amp;A</x:v>
+      </x:c>
+      <x:c r="E15" s="43" t="str">
+        <x:v>Published transcript</x:v>
+      </x:c>
+      <x:c r="F15" s="43" t="str">
+        <x:v>https://www.investing.com/news/transcripts/spacex-at-goldman-sachs-communacopia--technology-conference-2026-compute-push-93CH-4896834</x:v>
+      </x:c>
+      <x:c r="G15" s="43" t="str">
+        <x:v>Monetization and new hosting deal terms</x:v>
+      </x:c>
+      <x:c r="H15" s="43" t="str">
+        <x:v>Management claims</x:v>
+      </x:c>
+      <x:c r="I15" s="43" t="str">
+        <x:v>Use Q&amp;A; introductory summary misdates years; audio not reviewed</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="16">
+      <x:c r="A16" s="20" t="str">
+        <x:v>SRC-XAI-GS-EVENT-20260910</x:v>
+      </x:c>
+      <x:c r="B16" s="46" t="n">
+        <x:v>46275</x:v>
+      </x:c>
+      <x:c r="C16" s="20" t="str">
+        <x:v>SpaceX investor relations</x:v>
+      </x:c>
+      <x:c r="D16" s="44" t="str">
+        <x:v>Goldman Sachs Communacopia event</x:v>
+      </x:c>
+      <x:c r="E16" s="44" t="str">
+        <x:v>Issuer event page</x:v>
+      </x:c>
+      <x:c r="F16" s="44" t="str">
+        <x:v>https://ir.spacex.com/events/event-details/2026/Goldman-Sachs-2026-Communacopia-and-Technology-Conference-2026-u70jsP31xi/default.aspx</x:v>
+      </x:c>
+      <x:c r="G16" s="44" t="str">
+        <x:v>Event date and replay location</x:v>
+      </x:c>
+      <x:c r="H16" s="44" t="str">
+        <x:v>Primary</x:v>
+      </x:c>
+      <x:c r="I16" s="44" t="str">
+        <x:v>September 10 2026 12:25 PM PT; no financial figures on this page</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1ceb780fedb44566"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf7e17174ae05410f"/>
   </x:tableParts>
 </x:worksheet>
 </file>

</xml_diff>

<commit_message>
Review Oracle Q1 FY2027 compute economics and financing; preserve unresolved MW inputs
</commit_message>
<xml_diff>
--- a/data/ai-compute-economics.xlsx
+++ b/data/ai-compute-economics.xlsx
@@ -2,13 +2,13 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R1e62ba5d08a44ce7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Company Models" sheetId="2" r:id="R8b00635d9fc44b9c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Methods" sheetId="3" r:id="Re6620be9f68447b6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Token Economics" sheetId="4" r:id="R7267c0535ffb48d9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Benchmarks" sheetId="5" r:id="Rd0b70d9d56e7403c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="6" r:id="Rdf125edc0fcd412a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Read Me" sheetId="7" r:id="R1b81a77c6f0c4873"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="Rbd64e12deed04914"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Company Models" sheetId="2" r:id="Ree35e0c9756943a2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Methods" sheetId="3" r:id="R791fdb226e824c2f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Token Economics" sheetId="4" r:id="R8f89aab5a5174e20"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Benchmarks" sheetId="5" r:id="Ra9a35ab754cf4648"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="6" r:id="R58f065f00f6a455d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Read Me" sheetId="7" r:id="R1f873ac222864fd9"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -362,7 +362,7 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="SourceRegisterTable" displayName="SourceRegisterTable" ref="A4:I16" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="SourceRegisterTable" displayName="SourceRegisterTable" ref="A4:I29" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="9">
     <x:tableColumn id="1" name="Source ID"/>
     <x:tableColumn id="2" name="Date"/>
@@ -863,7 +863,7 @@
       </x:c>
       <x:c r="D17" s="19" t="str">
         <x:f>'Company Models'!N9</x:f>
-        <x:v>OPEN</x:v>
+        <x:v>PARTIAL</x:v>
       </x:c>
       <x:c r="E17" s="58" t="str">
         <x:f>IF('Company Models'!S9="","",'Company Models'!S9)</x:f>
@@ -1122,7 +1122,7 @@
     <x:col min="10" max="10" width="11" hidden="0" customWidth="1"/>
     <x:col min="11" max="11" width="12" hidden="0" customWidth="1"/>
     <x:col min="12" max="12" width="11" hidden="0" customWidth="1"/>
-    <x:col min="13" max="13" width="18" hidden="0" customWidth="1"/>
+    <x:col min="13" max="13" width="30" hidden="0" customWidth="1"/>
     <x:col min="14" max="14" width="15" hidden="0" customWidth="1"/>
     <x:col min="15" max="15" width="48" hidden="0" customWidth="1"/>
     <x:col min="16" max="16" width="21" hidden="0" customWidth="1"/>
@@ -1430,10 +1430,14 @@
         <x:v>SEGMENT-OCI</x:v>
       </x:c>
       <x:c r="C9" s="19" t="str">
-        <x:v>Open</x:v>
-      </x:c>
-      <x:c r="D9" s="27"/>
-      <x:c r="E9" s="29"/>
+        <x:v>Q1 FY2027</x:v>
+      </x:c>
+      <x:c r="D9" s="27" t="n">
+        <x:v>7400000000</x:v>
+      </x:c>
+      <x:c r="E9" s="29" t="n">
+        <x:v>4</x:v>
+      </x:c>
       <x:c r="F9" s="31"/>
       <x:c r="G9" s="33"/>
       <x:c r="H9" s="23"/>
@@ -1442,13 +1446,13 @@
       <x:c r="K9" s="35"/>
       <x:c r="L9" s="35"/>
       <x:c r="M9" s="19" t="str">
-        <x:v>SRC-CHAT-001</x:v>
+        <x:v>SRC-ORCL-Q1FY27-20260910</x:v>
       </x:c>
       <x:c r="N9" s="19" t="str">
-        <x:v>OPEN</x:v>
+        <x:v>PARTIAL</x:v>
       </x:c>
       <x:c r="O9" s="43" t="str">
-        <x:v>Needs OCI compute revenue and average active MW; RPO alone prohibited</x:v>
+        <x:v>IaaS only; AI share and average IT MW missing. 850MW additions excluded; PUE undisclosed.</x:v>
       </x:c>
       <x:c r="P9" s="37" t="str">
         <x:f>IF(OR(D9="",E9="",F9=""),"",D9*E9*F9)</x:f>
@@ -2066,16 +2070,16 @@
         <x:v>Hyperscaler</x:v>
       </x:c>
       <x:c r="D9" s="43" t="str">
-        <x:v>Annualized OCI or IaaS compute revenue adjusted for customer-supplied hardware</x:v>
+        <x:v>Recognized AI compute within OCI less hardware pass-through</x:v>
       </x:c>
       <x:c r="E9" s="43" t="str">
-        <x:v>Average effective utilized OCI IT MW</x:v>
+        <x:v>Time-weighted active AI IT MW and matching utilization</x:v>
       </x:c>
       <x:c r="F9" s="43" t="str">
-        <x:v>RPO is not period revenue; identify GPU pass-through</x:v>
+        <x:v>Exclude RPO and prepayment cash; no use of capacity additions as denominator</x:v>
       </x:c>
       <x:c r="G9" s="43" t="str">
-        <x:v>Configured; inputs open</x:v>
+        <x:v>Partial 2026-09-11; PUE not disclosed</x:v>
       </x:c>
     </x:row>
     <x:row r="10">
@@ -2265,7 +2269,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc16d947a88b04b35"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc11a2e38430743b8"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2889,7 +2893,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rcd47c55e6d8340dd"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc0e0b173d0b44852"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3293,7 +3297,7 @@
   </x:sheetPr>
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
-    <x:col min="1" max="1" width="24" hidden="0" customWidth="1"/>
+    <x:col min="1" max="1" width="34" hidden="0" customWidth="1"/>
     <x:col min="2" max="2" width="13" hidden="0" customWidth="1"/>
     <x:col min="3" max="3" width="24" hidden="0" customWidth="1"/>
     <x:col min="4" max="4" width="38" hidden="0" customWidth="1"/>
@@ -3675,38 +3679,415 @@
       </x:c>
     </x:row>
     <x:row r="16">
-      <x:c r="A16" s="20" t="str">
+      <x:c r="A16" s="19" t="str">
         <x:v>SRC-XAI-GS-EVENT-20260910</x:v>
       </x:c>
-      <x:c r="B16" s="46" t="n">
+      <x:c r="B16" s="45" t="n">
         <x:v>46275</x:v>
       </x:c>
-      <x:c r="C16" s="20" t="str">
+      <x:c r="C16" s="19" t="str">
         <x:v>SpaceX investor relations</x:v>
       </x:c>
-      <x:c r="D16" s="44" t="str">
+      <x:c r="D16" s="43" t="str">
         <x:v>Goldman Sachs Communacopia event</x:v>
       </x:c>
-      <x:c r="E16" s="44" t="str">
+      <x:c r="E16" s="43" t="str">
         <x:v>Issuer event page</x:v>
       </x:c>
-      <x:c r="F16" s="44" t="str">
+      <x:c r="F16" s="43" t="str">
         <x:v>https://ir.spacex.com/events/event-details/2026/Goldman-Sachs-2026-Communacopia-and-Technology-Conference-2026-u70jsP31xi/default.aspx</x:v>
       </x:c>
-      <x:c r="G16" s="44" t="str">
+      <x:c r="G16" s="43" t="str">
         <x:v>Event date and replay location</x:v>
       </x:c>
-      <x:c r="H16" s="44" t="str">
+      <x:c r="H16" s="43" t="str">
         <x:v>Primary</x:v>
       </x:c>
-      <x:c r="I16" s="44" t="str">
+      <x:c r="I16" s="43" t="str">
         <x:v>September 10 2026 12:25 PM PT; no financial figures on this page</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="17">
+      <x:c r="A17" s="19" t="str">
+        <x:v>SRC-ORCL-Q1FY27-20260910</x:v>
+      </x:c>
+      <x:c r="B17" s="45" t="n">
+        <x:v>46275</x:v>
+      </x:c>
+      <x:c r="C17" s="19" t="str">
+        <x:v>Oracle / SEC</x:v>
+      </x:c>
+      <x:c r="D17" s="43" t="str">
+        <x:v>Q1 FY2027 earnings release and financial tables</x:v>
+      </x:c>
+      <x:c r="E17" s="43" t="str">
+        <x:v>8-K Exhibit 99.1</x:v>
+      </x:c>
+      <x:c r="F17" s="43" t="str">
+        <x:v>https://www.sec.gov/Archives/edgar/data/1341439/000119312526387905/orcl-ex99_1.htm</x:v>
+      </x:c>
+      <x:c r="G17" s="43" t="str">
+        <x:v>Oracle OCI 2026-09-11 review</x:v>
+      </x:c>
+      <x:c r="H17" s="43" t="str">
+        <x:v>primary_read</x:v>
+      </x:c>
+      <x:c r="I17" s="43" t="str">
+        <x:v>Opening highlights; financial tables pp. 4-5: Cash Flows, Free Cash Flow, Net Cash Outlay; notes (2)-(3)</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="18">
+      <x:c r="A18" s="19" t="str">
+        <x:v>SRC-ORCL-10K-FY26</x:v>
+      </x:c>
+      <x:c r="B18" s="45" t="n">
+        <x:v>46195</x:v>
+      </x:c>
+      <x:c r="C18" s="19" t="str">
+        <x:v>Oracle / SEC</x:v>
+      </x:c>
+      <x:c r="D18" s="43" t="str">
+        <x:v>FY2026 Form 10-K</x:v>
+      </x:c>
+      <x:c r="E18" s="43" t="str">
+        <x:v>10-K</x:v>
+      </x:c>
+      <x:c r="F18" s="43" t="str">
+        <x:v>https://www.sec.gov/Archives/edgar/data/1341439/000119312526277521/orcl-20260531.htm</x:v>
+      </x:c>
+      <x:c r="G18" s="43" t="str">
+        <x:v>Oracle OCI 2026-09-11 review</x:v>
+      </x:c>
+      <x:c r="H18" s="43" t="str">
+        <x:v>primary_read</x:v>
+      </x:c>
+      <x:c r="I18" s="43" t="str">
+        <x:v>Note 4 p.81; Note 9 pp.88-90; MD&amp;A p.55; Note 1 p.72</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="19">
+      <x:c r="A19" s="19" t="str">
+        <x:v>SRC-ORCL-10Q-Q3FY26</x:v>
+      </x:c>
+      <x:c r="B19" s="45" t="n">
+        <x:v>46092</x:v>
+      </x:c>
+      <x:c r="C19" s="19" t="str">
+        <x:v>Oracle / SEC</x:v>
+      </x:c>
+      <x:c r="D19" s="43" t="str">
+        <x:v>Q3 FY2026 Form 10-Q</x:v>
+      </x:c>
+      <x:c r="E19" s="43" t="str">
+        <x:v>10-Q</x:v>
+      </x:c>
+      <x:c r="F19" s="43" t="str">
+        <x:v>https://www.sec.gov/Archives/edgar/data/1341439/000119312526101045/orcl-20260228.htm</x:v>
+      </x:c>
+      <x:c r="G19" s="43" t="str">
+        <x:v>Oracle OCI 2026-09-11 review</x:v>
+      </x:c>
+      <x:c r="H19" s="43" t="str">
+        <x:v>primary_read</x:v>
+      </x:c>
+      <x:c r="I19" s="43" t="str">
+        <x:v>Note 6 pp.12-14: Leases, Other Commitments and Certain Contingencies</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="20">
+      <x:c r="A20" s="19" t="str">
+        <x:v>SRC-ORCL-CEO-20260612</x:v>
+      </x:c>
+      <x:c r="B20" s="45" t="n">
+        <x:v>46185</x:v>
+      </x:c>
+      <x:c r="C20" s="19" t="str">
+        <x:v>Oracle</x:v>
+      </x:c>
+      <x:c r="D20" s="43" t="str">
+        <x:v>From the Q4 Earnings Call: Driving Sustainable Growth Through Durable Differentiation</x:v>
+      </x:c>
+      <x:c r="E20" s="43" t="str">
+        <x:v>issuer_prepared_remarks</x:v>
+      </x:c>
+      <x:c r="F20" s="43" t="str">
+        <x:v>https://blogs.oracle.com/ceo/from-the-q4-earnings-call</x:v>
+      </x:c>
+      <x:c r="G20" s="43" t="str">
+        <x:v>Oracle OCI 2026-09-11 review</x:v>
+      </x:c>
+      <x:c r="H20" s="43" t="str">
+        <x:v>primary_read</x:v>
+      </x:c>
+      <x:c r="I20" s="43" t="str">
+        <x:v>Enabling scale while growing profitability; Accelerating delivery; five largest sites</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="21">
+      <x:c r="A21" s="19" t="str">
+        <x:v>SRC-ORCL-ESG-FY25</x:v>
+      </x:c>
+      <x:c r="B21" s="45" t="str">
+        <x:v>2026-02</x:v>
+      </x:c>
+      <x:c r="C21" s="19" t="str">
+        <x:v>Oracle</x:v>
+      </x:c>
+      <x:c r="D21" s="43" t="str">
+        <x:v>Environmental and Social Impact FY25 Datasheet Version 6</x:v>
+      </x:c>
+      <x:c r="E21" s="43" t="str">
+        <x:v>sustainability_report</x:v>
+      </x:c>
+      <x:c r="F21" s="43" t="str">
+        <x:v>https://www.oracle.com/it/a/ocom/docs/social-impact-datasheet.pdf</x:v>
+      </x:c>
+      <x:c r="G21" s="43" t="str">
+        <x:v>Oracle OCI 2026-09-11 review</x:v>
+      </x:c>
+      <x:c r="H21" s="43" t="str">
+        <x:v>primary_read</x:v>
+      </x:c>
+      <x:c r="I21" s="43" t="str">
+        <x:v>p.3 Energy and Renewables; p.6 footnotes vii-ix</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="22">
+      <x:c r="A22" s="19" t="str">
+        <x:v>SRC-ORCL-CARBON-20250630</x:v>
+      </x:c>
+      <x:c r="B22" s="45" t="n">
+        <x:v>45838</x:v>
+      </x:c>
+      <x:c r="C22" s="19" t="str">
+        <x:v>Oracle</x:v>
+      </x:c>
+      <x:c r="D22" s="43" t="str">
+        <x:v>OCI Carbon Emissions Analysis: power-based calculations</x:v>
+      </x:c>
+      <x:c r="E22" s="43" t="str">
+        <x:v>issuer_methodology</x:v>
+      </x:c>
+      <x:c r="F22" s="43" t="str">
+        <x:v>https://blogs.oracle.com/sustainability/oci-carbon-emissions-power-based-calculations</x:v>
+      </x:c>
+      <x:c r="G22" s="43" t="str">
+        <x:v>Oracle OCI 2026-09-11 review</x:v>
+      </x:c>
+      <x:c r="H22" s="43" t="str">
+        <x:v>primary_read</x:v>
+      </x:c>
+      <x:c r="I22" s="43" t="str">
+        <x:v>What are power-based emissions; reporting experience</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="23">
+      <x:c r="A23" s="19" t="str">
+        <x:v>SRC-ORCL-CARBON-202302</x:v>
+      </x:c>
+      <x:c r="B23" s="45" t="str">
+        <x:v>2023-02</x:v>
+      </x:c>
+      <x:c r="C23" s="19" t="str">
+        <x:v>Oracle</x:v>
+      </x:c>
+      <x:c r="D23" s="43" t="str">
+        <x:v>Technical Carbon Calculation Guidance v1.0</x:v>
+      </x:c>
+      <x:c r="E23" s="43" t="str">
+        <x:v>technical_brief</x:v>
+      </x:c>
+      <x:c r="F23" s="43" t="str">
+        <x:v>https://www.oracle.com/a/ocom/docs/corporate/technical-carbon-calculation-guidance.pdf</x:v>
+      </x:c>
+      <x:c r="G23" s="43" t="str">
+        <x:v>Oracle OCI 2026-09-11 review</x:v>
+      </x:c>
+      <x:c r="H23" s="43" t="str">
+        <x:v>primary_read</x:v>
+      </x:c>
+      <x:c r="I23" s="43" t="str">
+        <x:v>pp.4-6 carbon boundary and calculation methodology</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="24">
+      <x:c r="A24" s="19" t="str">
+        <x:v>SRC-ORCL-GREEN-CLOUD-20260911</x:v>
+      </x:c>
+      <x:c r="B24" s="45" t="n">
+        <x:v>46276</x:v>
+      </x:c>
+      <x:c r="C24" s="19" t="str">
+        <x:v>Oracle</x:v>
+      </x:c>
+      <x:c r="D24" s="43" t="str">
+        <x:v>Oracle Cloud sustainability</x:v>
+      </x:c>
+      <x:c r="E24" s="43" t="str">
+        <x:v>issuer_webpage</x:v>
+      </x:c>
+      <x:c r="F24" s="43" t="str">
+        <x:v>https://www.oracle.com/sustainability/green-cloud/</x:v>
+      </x:c>
+      <x:c r="G24" s="43" t="str">
+        <x:v>Oracle OCI 2026-09-11 review</x:v>
+      </x:c>
+      <x:c r="H24" s="43" t="str">
+        <x:v>primary_read</x:v>
+      </x:c>
+      <x:c r="I24" s="43" t="str">
+        <x:v>Clean cloud; Measurement; linked datasheets</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="25">
+      <x:c r="A25" s="19" t="str">
+        <x:v>SRC-OPENAI-ORACLE-20250722</x:v>
+      </x:c>
+      <x:c r="B25" s="45" t="n">
+        <x:v>45860</x:v>
+      </x:c>
+      <x:c r="C25" s="19" t="str">
+        <x:v>OpenAI</x:v>
+      </x:c>
+      <x:c r="D25" s="43" t="str">
+        <x:v>Stargate advances with 4.5 GW partnership with Oracle</x:v>
+      </x:c>
+      <x:c r="E25" s="43" t="str">
+        <x:v>counterparty_announcement</x:v>
+      </x:c>
+      <x:c r="F25" s="43" t="str">
+        <x:v>https://openai.com/index/stargate-advances-with-partnership-with-oracle/</x:v>
+      </x:c>
+      <x:c r="G25" s="43" t="str">
+        <x:v>Oracle OCI 2026-09-11 review</x:v>
+      </x:c>
+      <x:c r="H25" s="43" t="str">
+        <x:v>primary_read</x:v>
+      </x:c>
+      <x:c r="I25" s="43" t="str">
+        <x:v>Opening agreement; Abilene initial workloads</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="26">
+      <x:c r="A26" s="19" t="str">
+        <x:v>SRC-OPENAI-STARGATE-20250923</x:v>
+      </x:c>
+      <x:c r="B26" s="45" t="n">
+        <x:v>45923</x:v>
+      </x:c>
+      <x:c r="C26" s="19" t="str">
+        <x:v>OpenAI</x:v>
+      </x:c>
+      <x:c r="D26" s="43" t="str">
+        <x:v>Five new Stargate sites</x:v>
+      </x:c>
+      <x:c r="E26" s="43" t="str">
+        <x:v>counterparty_announcement</x:v>
+      </x:c>
+      <x:c r="F26" s="43" t="str">
+        <x:v>https://openai.com/index/five-new-stargate-sites/</x:v>
+      </x:c>
+      <x:c r="G26" s="43" t="str">
+        <x:v>Oracle OCI 2026-09-11 review</x:v>
+      </x:c>
+      <x:c r="H26" s="43" t="str">
+        <x:v>primary_read</x:v>
+      </x:c>
+      <x:c r="I26" s="43" t="str">
+        <x:v>Oracle partnership paragraphs; Wisconsin update</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="27">
+      <x:c r="A27" s="19" t="str">
+        <x:v>SRC-CRUSOE-ABILENE-20250521</x:v>
+      </x:c>
+      <x:c r="B27" s="45" t="n">
+        <x:v>45798</x:v>
+      </x:c>
+      <x:c r="C27" s="19" t="str">
+        <x:v>Crusoe</x:v>
+      </x:c>
+      <x:c r="D27" s="43" t="str">
+        <x:v>Second phase of USD15 billion Abilene joint venture</x:v>
+      </x:c>
+      <x:c r="E27" s="43" t="str">
+        <x:v>counterparty_project_financing</x:v>
+      </x:c>
+      <x:c r="F27" s="43" t="str">
+        <x:v>https://www.crusoe.ai/resources/newsroom/crusoe-blue-owl-capital-and-primary-digital-infrastructure-enter-joint-venture</x:v>
+      </x:c>
+      <x:c r="G27" s="43" t="str">
+        <x:v>Oracle OCI 2026-09-11 review</x:v>
+      </x:c>
+      <x:c r="H27" s="43" t="str">
+        <x:v>primary_read</x:v>
+      </x:c>
+      <x:c r="I27" s="43" t="str">
+        <x:v>Opening JV terms; phase schedule; cooling design</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="28">
+      <x:c r="A28" s="19" t="str">
+        <x:v>SRC-ORCL-REVOLVER-20260306</x:v>
+      </x:c>
+      <x:c r="B28" s="45" t="n">
+        <x:v>46092</x:v>
+      </x:c>
+      <x:c r="C28" s="19" t="str">
+        <x:v>Oracle / SEC</x:v>
+      </x:c>
+      <x:c r="D28" s="43" t="str">
+        <x:v>USD10 billion revolving credit agreement dated March 6 2026</x:v>
+      </x:c>
+      <x:c r="E28" s="43" t="str">
+        <x:v>10-Q Exhibit 10.17</x:v>
+      </x:c>
+      <x:c r="F28" s="43" t="str">
+        <x:v>https://www.sec.gov/Archives/edgar/data/1341439/000119312526101045/orcl-ex10_17.htm</x:v>
+      </x:c>
+      <x:c r="G28" s="43" t="str">
+        <x:v>Oracle OCI 2026-09-11 review</x:v>
+      </x:c>
+      <x:c r="H28" s="43" t="str">
+        <x:v>primary_read</x:v>
+      </x:c>
+      <x:c r="I28" s="43" t="str">
+        <x:v>Cover; sections 2.01, 2.08, 2.21 and 6.02</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="29">
+      <x:c r="A29" s="20" t="str">
+        <x:v>SRC-ORCL-Q1FY27-EVENT</x:v>
+      </x:c>
+      <x:c r="B29" s="46" t="n">
+        <x:v>46275</x:v>
+      </x:c>
+      <x:c r="C29" s="20" t="str">
+        <x:v>Oracle</x:v>
+      </x:c>
+      <x:c r="D29" s="44" t="str">
+        <x:v>Q1 FY27 earnings event</x:v>
+      </x:c>
+      <x:c r="E29" s="44" t="str">
+        <x:v>issuer_event</x:v>
+      </x:c>
+      <x:c r="F29" s="44" t="str">
+        <x:v>https://investor.oracle.com/events-and-presentations/event-details/2026/Q1-FY27-Earnings/default.aspx</x:v>
+      </x:c>
+      <x:c r="G29" s="44" t="str">
+        <x:v>Oracle OCI 2026-09-11 review</x:v>
+      </x:c>
+      <x:c r="H29" s="44" t="str">
+        <x:v>metadata_read_transcript_unavailable</x:v>
+      </x:c>
+      <x:c r="I29" s="44" t="str">
+        <x:v>Event date and webcast link; linked player returned no readable transcript</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf7e17174ae05410f"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9a664ebc5989414c"/>
   </x:tableParts>
 </x:worksheet>
 </file>

</xml_diff>

<commit_message>
Review CoreWeave Q2 compute economics and structured financing
</commit_message>
<xml_diff>
--- a/data/ai-compute-economics.xlsx
+++ b/data/ai-compute-economics.xlsx
@@ -2,13 +2,13 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="Rbd64e12deed04914"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Company Models" sheetId="2" r:id="Ree35e0c9756943a2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Methods" sheetId="3" r:id="R791fdb226e824c2f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Token Economics" sheetId="4" r:id="R8f89aab5a5174e20"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Benchmarks" sheetId="5" r:id="Ra9a35ab754cf4648"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="6" r:id="R58f065f00f6a455d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Read Me" sheetId="7" r:id="R1f873ac222864fd9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R31c4f4b9b00d4ab9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Company Models" sheetId="2" r:id="R49fc04845fc44ae8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Methods" sheetId="3" r:id="R8288f841dca0496c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Token Economics" sheetId="4" r:id="Rfe9e0885443d435d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Benchmarks" sheetId="5" r:id="R596c12a194584f1b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="6" r:id="R76e382eb87ab4a2d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Read Me" sheetId="7" r:id="Rc26c46b89db744b8"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -362,7 +362,7 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="SourceRegisterTable" displayName="SourceRegisterTable" ref="A4:I29" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="SourceRegisterTable" displayName="SourceRegisterTable" ref="A4:I38" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="9">
     <x:tableColumn id="1" name="Source ID"/>
     <x:tableColumn id="2" name="Date"/>
@@ -888,7 +888,7 @@
       </x:c>
       <x:c r="D18" s="19" t="str">
         <x:f>'Company Models'!N10</x:f>
-        <x:v>OPEN</x:v>
+        <x:v>PARTIAL</x:v>
       </x:c>
       <x:c r="E18" s="58" t="str">
         <x:f>IF('Company Models'!S10="","",'Company Models'!S10)</x:f>
@@ -1479,25 +1479,33 @@
         <x:v>MERCHANT-CRWV</x:v>
       </x:c>
       <x:c r="C10" s="19" t="str">
-        <x:v>Open</x:v>
-      </x:c>
-      <x:c r="D10" s="27"/>
-      <x:c r="E10" s="29"/>
+        <x:v>Q2 2026</x:v>
+      </x:c>
+      <x:c r="D10" s="27" t="n">
+        <x:v>2575000000</x:v>
+      </x:c>
+      <x:c r="E10" s="29" t="n">
+        <x:v>4</x:v>
+      </x:c>
       <x:c r="F10" s="31"/>
-      <x:c r="G10" s="33"/>
-      <x:c r="H10" s="23"/>
+      <x:c r="G10" s="33" t="n">
+        <x:v>1250</x:v>
+      </x:c>
+      <x:c r="H10" s="23" t="str">
+        <x:v>Facility power</x:v>
+      </x:c>
       <x:c r="I10" s="35"/>
       <x:c r="J10" s="35"/>
       <x:c r="K10" s="35"/>
       <x:c r="L10" s="35"/>
       <x:c r="M10" s="19" t="str">
-        <x:v>SRC-WB-CRWV-001</x:v>
+        <x:v>SRC-CRWV-Q2FY26-ER</x:v>
       </x:c>
       <x:c r="N10" s="19" t="str">
-        <x:v>OPEN</x:v>
+        <x:v>PARTIAL</x:v>
       </x:c>
       <x:c r="O10" s="43" t="str">
-        <x:v>Reconstruct period-average active MW and compute-only revenue</x:v>
+        <x:v>All-cloud revenue and modeled period-average active-power proxy; compute mix power boundary PUE and utilization remain missing so normalized output stays blank</x:v>
       </x:c>
       <x:c r="P10" s="37" t="str">
         <x:f>IF(OR(D10="",E10="",F10=""),"",D10*E10*F10)</x:f>
@@ -2099,10 +2107,10 @@
         <x:v>Weighted-average active IT MW times utilization</x:v>
       </x:c>
       <x:c r="F10" s="43" t="str">
-        <x:v>Remove non-compute services and reconstruct average MW from activation dates</x:v>
+        <x:v>Remove storage networking and software; reconstruct average capacity; resolve active-power boundary and PUE</x:v>
       </x:c>
       <x:c r="G10" s="43" t="str">
-        <x:v>Configured; inputs open</x:v>
+        <x:v>Partial 2026-09-12; canonical output open</x:v>
       </x:c>
     </x:row>
     <x:row r="11">
@@ -2269,7 +2277,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc11a2e38430743b8"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R473e72239eb340db"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2893,7 +2901,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc0e0b173d0b44852"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re014a0c2a70c4cd8"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4056,38 +4064,299 @@
       </x:c>
     </x:row>
     <x:row r="29">
-      <x:c r="A29" s="20" t="str">
+      <x:c r="A29" s="19" t="str">
         <x:v>SRC-ORCL-Q1FY27-EVENT</x:v>
       </x:c>
-      <x:c r="B29" s="46" t="n">
+      <x:c r="B29" s="45" t="n">
         <x:v>46275</x:v>
       </x:c>
-      <x:c r="C29" s="20" t="str">
+      <x:c r="C29" s="19" t="str">
         <x:v>Oracle</x:v>
       </x:c>
-      <x:c r="D29" s="44" t="str">
+      <x:c r="D29" s="43" t="str">
         <x:v>Q1 FY27 earnings event</x:v>
       </x:c>
-      <x:c r="E29" s="44" t="str">
+      <x:c r="E29" s="43" t="str">
         <x:v>issuer_event</x:v>
       </x:c>
-      <x:c r="F29" s="44" t="str">
+      <x:c r="F29" s="43" t="str">
         <x:v>https://investor.oracle.com/events-and-presentations/event-details/2026/Q1-FY27-Earnings/default.aspx</x:v>
       </x:c>
-      <x:c r="G29" s="44" t="str">
+      <x:c r="G29" s="43" t="str">
         <x:v>Oracle OCI 2026-09-11 review</x:v>
       </x:c>
-      <x:c r="H29" s="44" t="str">
+      <x:c r="H29" s="43" t="str">
         <x:v>metadata_read_transcript_unavailable</x:v>
       </x:c>
-      <x:c r="I29" s="44" t="str">
+      <x:c r="I29" s="43" t="str">
         <x:v>Event date and webcast link; linked player returned no readable transcript</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="30">
+      <x:c r="A30" s="19" t="str">
+        <x:v>SRC-CRWV-10K-FY25</x:v>
+      </x:c>
+      <x:c r="B30" s="45" t="n">
+        <x:v>46083</x:v>
+      </x:c>
+      <x:c r="C30" s="19" t="str">
+        <x:v>CoreWeave / SEC</x:v>
+      </x:c>
+      <x:c r="D30" s="43" t="str">
+        <x:v>FY2025 Form 10-K</x:v>
+      </x:c>
+      <x:c r="E30" s="43" t="str">
+        <x:v>10-K</x:v>
+      </x:c>
+      <x:c r="F30" s="43" t="str">
+        <x:v>https://www.sec.gov/Archives/edgar/data/1769628/000176962826000104/crwv-20251231.htm</x:v>
+      </x:c>
+      <x:c r="G30" s="43" t="str">
+        <x:v>CoreWeave 2026-09-12 review</x:v>
+      </x:c>
+      <x:c r="H30" s="43" t="str">
+        <x:v>primary_read</x:v>
+      </x:c>
+      <x:c r="I30" s="43" t="str">
+        <x:v>Item 1 pp.5-11; revenue pp.97-102; leases pp.111-112; debt pp.113-116</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="31">
+      <x:c r="A31" s="19" t="str">
+        <x:v>SRC-CRWV-10Q-Q2FY26</x:v>
+      </x:c>
+      <x:c r="B31" s="45" t="n">
+        <x:v>46246</x:v>
+      </x:c>
+      <x:c r="C31" s="19" t="str">
+        <x:v>CoreWeave / SEC</x:v>
+      </x:c>
+      <x:c r="D31" s="43" t="str">
+        <x:v>Q2 2026 Form 10-Q</x:v>
+      </x:c>
+      <x:c r="E31" s="43" t="str">
+        <x:v>10-Q</x:v>
+      </x:c>
+      <x:c r="F31" s="43" t="str">
+        <x:v>https://www.sec.gov/Archives/edgar/data/1769628/000176962826000366/crwv-20260630.htm</x:v>
+      </x:c>
+      <x:c r="G31" s="43" t="str">
+        <x:v>CoreWeave 2026-09-12 review</x:v>
+      </x:c>
+      <x:c r="H31" s="43" t="str">
+        <x:v>primary_read</x:v>
+      </x:c>
+      <x:c r="I31" s="43" t="str">
+        <x:v>Note 2 pp.14-15; Note 3 pp.15-17; Note 5 p.20; Note 9 pp.23-25; Note 10 pp.26-31; MD&amp;A pp.42-47</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="32">
+      <x:c r="A32" s="19" t="str">
+        <x:v>SRC-CRWV-Q1FY26-ER</x:v>
+      </x:c>
+      <x:c r="B32" s="45" t="n">
+        <x:v>46149</x:v>
+      </x:c>
+      <x:c r="C32" s="19" t="str">
+        <x:v>CoreWeave</x:v>
+      </x:c>
+      <x:c r="D32" s="43" t="str">
+        <x:v>CoreWeave Reports Strong First Quarter 2026 Results</x:v>
+      </x:c>
+      <x:c r="E32" s="43" t="str">
+        <x:v>issuer_earnings_release</x:v>
+      </x:c>
+      <x:c r="F32" s="43" t="str">
+        <x:v>https://investors.coreweave.com/news/news-details/2026/CoreWeave-Reports-Strong-First-Quarter-2026-Results/default.aspx</x:v>
+      </x:c>
+      <x:c r="G32" s="43" t="str">
+        <x:v>CoreWeave opening power and contracts</x:v>
+      </x:c>
+      <x:c r="H32" s="43" t="str">
+        <x:v>primary_read</x:v>
+      </x:c>
+      <x:c r="I32" s="43" t="str">
+        <x:v>Financial and power highlights; DDTL 4.0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="33">
+      <x:c r="A33" s="19" t="str">
+        <x:v>SRC-CRWV-Q2FY26-ER</x:v>
+      </x:c>
+      <x:c r="B33" s="45" t="n">
+        <x:v>46245</x:v>
+      </x:c>
+      <x:c r="C33" s="19" t="str">
+        <x:v>CoreWeave</x:v>
+      </x:c>
+      <x:c r="D33" s="43" t="str">
+        <x:v>CoreWeave Reports Strong Second Quarter 2026 Results</x:v>
+      </x:c>
+      <x:c r="E33" s="43" t="str">
+        <x:v>issuer_earnings_release</x:v>
+      </x:c>
+      <x:c r="F33" s="43" t="str">
+        <x:v>https://investors.coreweave.com/news/news-details/2026/CoreWeave-Reports-Strong-Second-Quarter-2026-Results/</x:v>
+      </x:c>
+      <x:c r="G33" s="43" t="str">
+        <x:v>CoreWeave Q2 revenue power and backlog</x:v>
+      </x:c>
+      <x:c r="H33" s="43" t="str">
+        <x:v>primary_read</x:v>
+      </x:c>
+      <x:c r="I33" s="43" t="str">
+        <x:v>Financial highlights; backlog footnote; active and contracted power</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="34">
+      <x:c r="A34" s="19" t="str">
+        <x:v>SRC-CRWV-DDTL55-8K</x:v>
+      </x:c>
+      <x:c r="B34" s="45" t="n">
+        <x:v>46244</x:v>
+      </x:c>
+      <x:c r="C34" s="19" t="str">
+        <x:v>CoreWeave / SEC</x:v>
+      </x:c>
+      <x:c r="D34" s="43" t="str">
+        <x:v>DDTL 5.5 Facility Form 8-K</x:v>
+      </x:c>
+      <x:c r="E34" s="43" t="str">
+        <x:v>8-K</x:v>
+      </x:c>
+      <x:c r="F34" s="43" t="str">
+        <x:v>https://www.sec.gov/Archives/edgar/data/1769628/000176962826000357/crwv-20260807.htm</x:v>
+      </x:c>
+      <x:c r="G34" s="43" t="str">
+        <x:v>CoreWeave DDTL 5.5</x:v>
+      </x:c>
+      <x:c r="H34" s="43" t="str">
+        <x:v>primary_read</x:v>
+      </x:c>
+      <x:c r="I34" s="43" t="str">
+        <x:v>Item 1.01 amount use maturity pricing guarantees collateral and DSCR</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="35">
+      <x:c r="A35" s="19" t="str">
+        <x:v>SRC-CRWV-DDTL55-EX10</x:v>
+      </x:c>
+      <x:c r="B35" s="45" t="n">
+        <x:v>46241</x:v>
+      </x:c>
+      <x:c r="C35" s="19" t="str">
+        <x:v>CoreWeave / SEC</x:v>
+      </x:c>
+      <x:c r="D35" s="43" t="str">
+        <x:v>DDTL 5.5 Credit Agreement</x:v>
+      </x:c>
+      <x:c r="E35" s="43" t="str">
+        <x:v>8-K Exhibit 10.1</x:v>
+      </x:c>
+      <x:c r="F35" s="43" t="str">
+        <x:v>https://www.sec.gov/Archives/edgar/data/1769628/000176962826000357/ex101creditagreement.htm</x:v>
+      </x:c>
+      <x:c r="G35" s="43" t="str">
+        <x:v>CoreWeave DDTL 5.5 terms</x:v>
+      </x:c>
+      <x:c r="H35" s="43" t="str">
+        <x:v>primary_read</x:v>
+      </x:c>
+      <x:c r="I35" s="43" t="str">
+        <x:v>Definitions and sections 2.01 2.06 2.08-2.11</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="36">
+      <x:c r="A36" s="19" t="str">
+        <x:v>SRC-CRWV-DDTL55-GUARANTEE</x:v>
+      </x:c>
+      <x:c r="B36" s="45" t="n">
+        <x:v>46241</x:v>
+      </x:c>
+      <x:c r="C36" s="19" t="str">
+        <x:v>CoreWeave / SEC</x:v>
+      </x:c>
+      <x:c r="D36" s="43" t="str">
+        <x:v>DDTL 5.5 Parent Guarantee and Pledge Agreement</x:v>
+      </x:c>
+      <x:c r="E36" s="43" t="str">
+        <x:v>8-K Exhibit 10.2</x:v>
+      </x:c>
+      <x:c r="F36" s="43" t="str">
+        <x:v>https://www.sec.gov/Archives/edgar/data/1769628/000176962826000357/ex102parentguarantee.htm</x:v>
+      </x:c>
+      <x:c r="G36" s="43" t="str">
+        <x:v>CoreWeave DDTL 5.5 guarantee</x:v>
+      </x:c>
+      <x:c r="H36" s="43" t="str">
+        <x:v>primary_read</x:v>
+      </x:c>
+      <x:c r="I36" s="43" t="str">
+        <x:v>Section 2.1 unconditional and irrevocable guarantee</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="37">
+      <x:c r="A37" s="19" t="str">
+        <x:v>SRC-CRWV-DDTL50-20260518</x:v>
+      </x:c>
+      <x:c r="B37" s="45" t="n">
+        <x:v>46160</x:v>
+      </x:c>
+      <x:c r="C37" s="19" t="str">
+        <x:v>CoreWeave</x:v>
+      </x:c>
+      <x:c r="D37" s="43" t="str">
+        <x:v>CoreWeave Closes USD3.1 Billion Loan Facility</x:v>
+      </x:c>
+      <x:c r="E37" s="43" t="str">
+        <x:v>issuer_financing_release</x:v>
+      </x:c>
+      <x:c r="F37" s="43" t="str">
+        <x:v>https://investors.coreweave.com/news/news-details/2026/CoreWeave-Closes-3-1-Billion-Loan-Facility-Expanding-Access-to-Public-Markets-for-GPU-Backed-Financing/</x:v>
+      </x:c>
+      <x:c r="G37" s="43" t="str">
+        <x:v>CoreWeave DDTL 5.0</x:v>
+      </x:c>
+      <x:c r="H37" s="43" t="str">
+        <x:v>primary_read</x:v>
+      </x:c>
+      <x:c r="I37" s="43" t="str">
+        <x:v>Two non-investment-grade customer contracts; SOFR plus 4.50%; approximately 5.5 years</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="38">
+      <x:c r="A38" s="20" t="str">
+        <x:v>SRC-CRWV-META-20260409</x:v>
+      </x:c>
+      <x:c r="B38" s="46" t="n">
+        <x:v>46121</x:v>
+      </x:c>
+      <x:c r="C38" s="20" t="str">
+        <x:v>CoreWeave</x:v>
+      </x:c>
+      <x:c r="D38" s="44" t="str">
+        <x:v>CoreWeave and Meta Announce USD21 Billion Expanded AI Infrastructure Agreement</x:v>
+      </x:c>
+      <x:c r="E38" s="44" t="str">
+        <x:v>issuer_customer_agreement</x:v>
+      </x:c>
+      <x:c r="F38" s="44" t="str">
+        <x:v>https://investors.coreweave.com/news/news-details/2026/CoreWeave-and-Meta-Announce-21-Billion-Expanded-AI-Infrastructure-Agreement/default.aspx</x:v>
+      </x:c>
+      <x:c r="G38" s="44" t="str">
+        <x:v>CoreWeave Meta agreement</x:v>
+      </x:c>
+      <x:c r="H38" s="44" t="str">
+        <x:v>primary_read</x:v>
+      </x:c>
+      <x:c r="I38" s="44" t="str">
+        <x:v>Dedicated multi-location capacity through December 2032; initial Vera Rubin deployments</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9a664ebc5989414c"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf3fab472898a49ce"/>
   </x:tableParts>
 </x:worksheet>
 </file>

</xml_diff>